<commit_message>
tambah menu anallytiticx, pekerjaan oh, dan perbaikan dashboard
</commit_message>
<xml_diff>
--- a/storage/templates/TEMPLATE-IMPORT-ALAT.xlsx
+++ b/storage/templates/TEMPLATE-IMPORT-ALAT.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="120">
   <si>
     <t>Nama</t>
   </si>
@@ -93,6 +93,9 @@
   </si>
   <si>
     <t>Digital Micrometer Mitutoyo digital micrometer head metric 350-252-30 25/0.001 mm</t>
+  </si>
+  <si>
+    <t>Max Demand (opsional)</t>
   </si>
   <si>
     <t>Jenis Tools</t>
@@ -742,7 +745,7 @@
   <sheetPr filterMode="1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="50.90625" customWidth="true" style="0"/>
@@ -750,9 +753,10 @@
     <col min="3" max="3" width="14.81640625" customWidth="true" style="0"/>
     <col min="6" max="6" width="22" customWidth="true" style="0"/>
     <col min="7" max="7" width="20" customWidth="true" style="0"/>
+    <col min="8" max="8" width="22" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" customHeight="1" ht="15.5" s="1" customFormat="1">
+    <row r="1" spans="1:8" customHeight="1" ht="15.5" s="1" customFormat="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -774,8 +778,11 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
@@ -796,7 +803,7 @@
       </c>
       <c r="G2" s="3"/>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:8">
       <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
@@ -817,7 +824,7 @@
       </c>
       <c r="G3" s="3"/>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:8">
       <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
@@ -838,7 +845,7 @@
       </c>
       <c r="G4" s="3"/>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:8">
       <c r="A5" s="3" t="s">
         <v>17</v>
       </c>
@@ -859,7 +866,7 @@
       </c>
       <c r="G5" s="3"/>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:8">
       <c r="A6" s="3" t="s">
         <v>18</v>
       </c>
@@ -880,7 +887,7 @@
       </c>
       <c r="G6" s="3"/>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:8">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -901,7 +908,7 @@
       </c>
       <c r="G7" s="3"/>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:8">
       <c r="A8" s="3" t="s">
         <v>24</v>
       </c>
@@ -944,10 +951,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -960,7 +967,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
         <v>15</v>
@@ -968,7 +975,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
@@ -976,307 +983,307 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -1286,37 +1293,37 @@
     </row>
     <row r="67" spans="1:2">
       <c r="A67" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -1326,112 +1333,112 @@
     </row>
     <row r="75" spans="1:2">
       <c r="A75" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>